<commit_message>
community analysis updated and better
</commit_message>
<xml_diff>
--- a/backend/analysis_report.xlsx
+++ b/backend/analysis_report.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,7 +446,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>disease</t>
+          <t>health_issue</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -832,6 +832,158 @@
       </c>
       <c r="H11" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>50</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Abuja</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Typhoid</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Fever;Headache</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>30</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Kano</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Cholera</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Vomiting;Diarrhea</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>34</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Ibadan</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Malaria</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Fever;Chills</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>22</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Typhoid</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Fever;Headache</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>